<commit_message>
Updated sample docs formatting and templates
</commit_message>
<xml_diff>
--- a/Analysis Examples/Account-Roll-Forward-Analysis.xlsx
+++ b/Analysis Examples/Account-Roll-Forward-Analysis.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roll Forward" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roll Forward Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roll Forward Analysis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roll Forward" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roll Forward'!$A$2:$X$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Roll Forward'!$A$2:$X$2</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -79,7 +79,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -161,6 +161,56 @@
         <fgColor rgb="FFFFF0DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCDD2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -192,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -268,6 +318,52 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,6 +625,592 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C44"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="15.75"/>
+  <cols>
+    <col width="28" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="52" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>REPORT SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Report Generated</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Wednesday, April 22, 2026, 5:21 PM</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Current (End) Period</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>2016-08-27</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Most recent period in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Dataset Period Range</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>2015-08-29 through 2016-08-27</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>13 fiscal periods</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>GLOK Baseline Period</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2015-08-29</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Earliest period loaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>VarOK Baseline Date</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2021-05-27 13:07:51</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Date RapidReconciler was last reset</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>2 (00010, 00050)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Co. 10 = 14 accounts; Co. 50 = 1 account</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Accounts (Unique)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Distinct LongAccount values</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Total Data Rows</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>15 accounts x 13 periods</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>GLOK = "no" Rows</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>No GL roll forward breaks detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>VarOK = "no" Rows</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>No variance roll forward breaks detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>End Period Total EndGL</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>$18,724,064.22</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Sum of all accounts, current period</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>End Period Total Perpetual</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>$18,710,860.69</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Sum of all accounts, current period</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>End Period UnpostBatch</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>No unposted batches in current period</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="25" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>ROW COLOR KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Criteria</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Row Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>GLOK = "no" OR VarOK = "no" — roll forward break</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>GLOK = "end" with non-zero UnpostBatch</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="44" t="inlineStr">
+        <is>
+          <t>Light Yellow</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>GLOK = "yes" with non-zero UnpostBatch — historical with pending batches</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="43" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>GLOK = "end" with zero UnpostBatch — current period, clean</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>White/Gray</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>All other rows (baseline or clean historical)</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="25" t="n"/>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="25" t="n"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>GL ROLL FORWARD (GLOK) FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="37.5" customHeight="1">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>No GLOK = "no" rows were found in this export. All 195 rows carry the baseline, yes, or end designation. The GL balance rolled forward without interruption across all 13 periods for all 15 accounts in both companies. No corrective action is required for GL continuity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="25" t="n"/>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>VARIANCE ROLL FORWARD (VarOK) FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="37.5" customHeight="1">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>No VarOK = "no" rows were found in this export. The variance chain is intact across all periods for all accounts. The VarOK baseline date (2021-05-27) post-dating the dataset start (2015-08-29) is expected — it reflects a RapidReconciler reset after initial data load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="25" t="n"/>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="25" t="n"/>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>HISTORICAL UNPOSTED BATCH SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LongAccount</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>EndGL | UnpostBatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>No accounts in any historical period have a non-zero UnpostBatch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="37.5" customHeight="1">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>Covers all periods except the current (end) period. A non-zero UnpostBatch in a historical period indicates a batch was approved but unposted at period-end and posted retroactively, which would have caused GLOK = "no" in the following period. In this export no historical unposted batches are present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="25" t="n"/>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="25" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>PERIOD VARIANCE BY ACCOUNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>LongAccount</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Variance | OOB | UnpostBatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>5000000.145000</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>2016-07-30</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Var: -$262.43  OOB: -$18,674.74  UnpostBatch: $0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="37.5" customHeight="1">
+      <c r="A39" s="48" t="inlineStr">
+        <is>
+          <t>Covers the prior 3 periods only (2016-05-28, 2016-07-02, 2016-07-30). Rows are shown where OOB absolute value exceeds $100 or UnpostBatch is non-zero. JE amounts and CardexVar are excluded from this section. OOB in these periods is informational; escalate only if accompanied by a VarOK = "no" flag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="25" t="n"/>
+      <c r="B40" s="25" t="n"/>
+      <c r="C40" s="25" t="n"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>RECOMMENDED ACTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="112" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>1 — High</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>Investigate OOB on 5000000.145000 (Company 50, GBP) in 2016-07-30: OOB of -$18,674.74 exceeds the $100 threshold in a closed historical period. Query F0902 and F0911 for this account and period to confirm the discrepancy. If confirmed, run R099102 in proof mode then final mode to resync F0902 from F0911. Involve your JD Edwards administrator before running in final mode.</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Cost Accountant / JD Edwards Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="70" customHeight="1">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>2 — Informational</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>No GL roll forward breaks (GLOK = "no") and no variance roll forward breaks (VarOK = "no") were detected. No batch posting or R099102 is required for continuity. Confirm this remains true at the next RapidReconciler refresh.</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Cost Accountant</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A26:C26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:X197"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="15.75"/>
   <cols>
@@ -1797,95 +2479,96 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C15" s="39" t="inlineStr">
         <is>
           <t>00223829</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D15" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.CC            </t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
+      <c r="E15" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F15" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="23" t="n">
+      <c r="F15" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="40" t="n">
         <v>105711.68</v>
       </c>
-      <c r="H15" s="23" t="n">
+      <c r="H15" s="40" t="n">
         <v>-5201.24</v>
       </c>
-      <c r="I15" s="23" t="n">
+      <c r="I15" s="40" t="n">
         <v>100510.44</v>
       </c>
-      <c r="J15" s="22" t="inlineStr">
+      <c r="J15" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K15" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="23" t="n">
+      <c r="K15" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="40" t="n">
         <v>-5201.18</v>
       </c>
-      <c r="M15" s="23" t="n">
+      <c r="M15" s="40" t="n">
         <v>100399.57</v>
       </c>
-      <c r="N15" s="23" t="n">
+      <c r="N15" s="40" t="n">
         <v>0.01</v>
       </c>
-      <c r="O15" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="23" t="n">
+      <c r="O15" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="40" t="n">
         <v>0.06</v>
       </c>
-      <c r="Q15" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="23" t="n">
+      <c r="Q15" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="40" t="n">
         <v>110.87</v>
       </c>
-      <c r="S15" s="23" t="n">
+      <c r="S15" s="40" t="n">
         <v>110.92</v>
       </c>
-      <c r="T15" s="22" t="inlineStr">
+      <c r="T15" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U15" s="22" t="inlineStr">
+      <c r="U15" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V15" s="22" t="inlineStr">
+      <c r="V15" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W15" s="22" t="inlineStr">
+      <c r="W15" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">CC      </t>
         </is>
       </c>
+      <c r="X15" s="41" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2980,95 +3663,96 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C28" s="22" t="inlineStr">
+      <c r="C28" s="39" t="inlineStr">
         <is>
           <t>00223837</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.FM            </t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
+      <c r="E28" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F28" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="23" t="n">
+      <c r="F28" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="40" t="n">
         <v>23753.48</v>
       </c>
-      <c r="H28" s="23" t="n">
+      <c r="H28" s="40" t="n">
         <v>15897.35</v>
       </c>
-      <c r="I28" s="23" t="n">
+      <c r="I28" s="40" t="n">
         <v>39650.83</v>
       </c>
-      <c r="J28" s="22" t="inlineStr">
+      <c r="J28" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="23" t="n">
+      <c r="K28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="40" t="n">
         <v>15897.35</v>
       </c>
-      <c r="M28" s="23" t="n">
+      <c r="M28" s="40" t="n">
         <v>39650.83</v>
       </c>
-      <c r="N28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="22" t="inlineStr">
+      <c r="N28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U28" s="22" t="inlineStr">
+      <c r="U28" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V28" s="22" t="inlineStr">
+      <c r="V28" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W28" s="22" t="inlineStr">
+      <c r="W28" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">FM      </t>
         </is>
       </c>
+      <c r="X28" s="41" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4163,95 +4847,96 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="inlineStr">
+      <c r="A41" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C41" s="39" t="inlineStr">
         <is>
           <t>00223845</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.MM            </t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E41" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F41" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="23" t="n">
+      <c r="F41" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="40" t="n">
         <v>671149.09</v>
       </c>
-      <c r="H41" s="23" t="n">
+      <c r="H41" s="40" t="n">
         <v>-45917.31</v>
       </c>
-      <c r="I41" s="23" t="n">
+      <c r="I41" s="40" t="n">
         <v>625231.78</v>
       </c>
-      <c r="J41" s="22" t="inlineStr">
+      <c r="J41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="23" t="n">
+      <c r="K41" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="40" t="n">
         <v>-45917.33</v>
       </c>
-      <c r="M41" s="23" t="n">
+      <c r="M41" s="40" t="n">
         <v>625085.49</v>
       </c>
-      <c r="N41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="23" t="n">
+      <c r="N41" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="40" t="n">
         <v>-0.02</v>
       </c>
-      <c r="Q41" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="23" t="n">
+      <c r="Q41" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="40" t="n">
         <v>146.29</v>
       </c>
-      <c r="S41" s="23" t="n">
+      <c r="S41" s="40" t="n">
         <v>146.27</v>
       </c>
-      <c r="T41" s="22" t="inlineStr">
+      <c r="T41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U41" s="22" t="inlineStr">
+      <c r="U41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V41" s="22" t="inlineStr">
+      <c r="V41" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W41" s="22" t="inlineStr">
+      <c r="W41" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">MM      </t>
         </is>
       </c>
+      <c r="X41" s="41" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5346,95 +6031,96 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="A54" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B54" s="22" t="inlineStr">
+      <c r="B54" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C54" s="22" t="inlineStr">
+      <c r="C54" s="39" t="inlineStr">
         <is>
           <t>00223853</t>
         </is>
       </c>
-      <c r="D54" s="22" t="inlineStr">
+      <c r="D54" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.PM            </t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr">
+      <c r="E54" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F54" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="22" t="inlineStr">
+      <c r="F54" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="S54" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="T54" s="22" t="inlineStr">
+      <c r="K54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S54" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T54" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U54" s="22" t="inlineStr">
+      <c r="U54" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V54" s="22" t="inlineStr">
+      <c r="V54" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W54" s="22" t="inlineStr">
+      <c r="W54" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">PM      </t>
         </is>
       </c>
+      <c r="X54" s="41" t="n"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6529,95 +7215,96 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="22" t="inlineStr">
+      <c r="A67" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B67" s="22" t="inlineStr">
+      <c r="B67" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C67" s="22" t="inlineStr">
+      <c r="C67" s="39" t="inlineStr">
         <is>
           <t>00223861</t>
         </is>
       </c>
-      <c r="D67" s="22" t="inlineStr">
+      <c r="D67" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.RW            </t>
         </is>
       </c>
-      <c r="E67" s="22" t="inlineStr">
+      <c r="E67" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F67" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" s="23" t="n">
+      <c r="F67" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="40" t="n">
         <v>328521.2</v>
       </c>
-      <c r="H67" s="23" t="n">
+      <c r="H67" s="40" t="n">
         <v>8258.66</v>
       </c>
-      <c r="I67" s="23" t="n">
+      <c r="I67" s="40" t="n">
         <v>336779.86</v>
       </c>
-      <c r="J67" s="22" t="inlineStr">
+      <c r="J67" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K67" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L67" s="23" t="n">
+      <c r="K67" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" s="40" t="n">
         <v>8258.66</v>
       </c>
-      <c r="M67" s="23" t="n">
+      <c r="M67" s="40" t="n">
         <v>335396.47</v>
       </c>
-      <c r="N67" s="23" t="n">
+      <c r="N67" s="40" t="n">
         <v>0.02</v>
       </c>
-      <c r="O67" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P67" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q67" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R67" s="23" t="n">
+      <c r="O67" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" s="40" t="n">
         <v>1383.39</v>
       </c>
-      <c r="S67" s="23" t="n">
+      <c r="S67" s="40" t="n">
         <v>1383.37</v>
       </c>
-      <c r="T67" s="22" t="inlineStr">
+      <c r="T67" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U67" s="22" t="inlineStr">
+      <c r="U67" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V67" s="22" t="inlineStr">
+      <c r="V67" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W67" s="22" t="inlineStr">
+      <c r="W67" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">RW      </t>
         </is>
       </c>
+      <c r="X67" s="41" t="n"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7712,95 +8399,96 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="22" t="inlineStr">
+      <c r="A80" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B80" s="22" t="inlineStr">
+      <c r="B80" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C80" s="22" t="inlineStr">
+      <c r="C80" s="39" t="inlineStr">
         <is>
           <t>00223870</t>
         </is>
       </c>
-      <c r="D80" s="22" t="inlineStr">
+      <c r="D80" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.141000.SM            </t>
         </is>
       </c>
-      <c r="E80" s="22" t="inlineStr">
+      <c r="E80" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F80" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G80" s="23" t="n">
+      <c r="F80" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="40" t="n">
         <v>1105003.17</v>
       </c>
-      <c r="H80" s="23" t="n">
+      <c r="H80" s="40" t="n">
         <v>34812.3</v>
       </c>
-      <c r="I80" s="23" t="n">
+      <c r="I80" s="40" t="n">
         <v>1139815.47</v>
       </c>
-      <c r="J80" s="22" t="inlineStr">
+      <c r="J80" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K80" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L80" s="23" t="n">
+      <c r="K80" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" s="40" t="n">
         <v>34812.29</v>
       </c>
-      <c r="M80" s="23" t="n">
+      <c r="M80" s="40" t="n">
         <v>1132569.28</v>
       </c>
-      <c r="N80" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O80" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P80" s="23" t="n">
+      <c r="N80" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O80" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P80" s="40" t="n">
         <v>-0.01</v>
       </c>
-      <c r="Q80" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R80" s="23" t="n">
+      <c r="Q80" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" s="40" t="n">
         <v>7246.19</v>
       </c>
-      <c r="S80" s="23" t="n">
+      <c r="S80" s="40" t="n">
         <v>7246.18</v>
       </c>
-      <c r="T80" s="22" t="inlineStr">
+      <c r="T80" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U80" s="22" t="inlineStr">
+      <c r="U80" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V80" s="22" t="inlineStr">
+      <c r="V80" s="39" t="inlineStr">
         <is>
           <t>141000</t>
         </is>
       </c>
-      <c r="W80" s="22" t="inlineStr">
+      <c r="W80" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">SM      </t>
         </is>
       </c>
+      <c r="X80" s="41" t="n"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8895,95 +9583,96 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="22" t="inlineStr">
+      <c r="A93" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B93" s="22" t="inlineStr">
+      <c r="B93" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C93" s="22" t="inlineStr">
+      <c r="C93" s="39" t="inlineStr">
         <is>
           <t>00223888</t>
         </is>
       </c>
-      <c r="D93" s="22" t="inlineStr">
+      <c r="D93" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.142000               </t>
         </is>
       </c>
-      <c r="E93" s="22" t="inlineStr">
+      <c r="E93" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F93" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G93" s="23" t="n">
+      <c r="F93" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="40" t="n">
         <v>8258329.04</v>
       </c>
-      <c r="H93" s="23" t="n">
+      <c r="H93" s="40" t="n">
         <v>138087.88</v>
       </c>
-      <c r="I93" s="23" t="n">
+      <c r="I93" s="40" t="n">
         <v>8396416.92</v>
       </c>
-      <c r="J93" s="22" t="inlineStr">
+      <c r="J93" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K93" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L93" s="23" t="n">
+      <c r="K93" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" s="40" t="n">
         <v>137389.03</v>
       </c>
-      <c r="M93" s="23" t="n">
+      <c r="M93" s="40" t="n">
         <v>8391759</v>
       </c>
-      <c r="N93" s="23" t="n">
+      <c r="N93" s="40" t="n">
         <v>0.01</v>
       </c>
-      <c r="O93" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P93" s="23" t="n">
+      <c r="O93" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P93" s="40" t="n">
         <v>-698.85</v>
       </c>
-      <c r="Q93" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R93" s="23" t="n">
+      <c r="Q93" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" s="40" t="n">
         <v>4657.92</v>
       </c>
-      <c r="S93" s="23" t="n">
+      <c r="S93" s="40" t="n">
         <v>3959.06</v>
       </c>
-      <c r="T93" s="22" t="inlineStr">
+      <c r="T93" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U93" s="22" t="inlineStr">
+      <c r="U93" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V93" s="22" t="inlineStr">
+      <c r="V93" s="39" t="inlineStr">
         <is>
           <t>142000</t>
         </is>
       </c>
-      <c r="W93" s="22" t="inlineStr">
+      <c r="W93" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
+      <c r="X93" s="41" t="n"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10078,95 +10767,96 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="22" t="inlineStr">
+      <c r="A106" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B106" s="22" t="inlineStr">
+      <c r="B106" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C106" s="22" t="inlineStr">
+      <c r="C106" s="39" t="inlineStr">
         <is>
           <t>00223917</t>
         </is>
       </c>
-      <c r="D106" s="22" t="inlineStr">
+      <c r="D106" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143000.MLD           </t>
         </is>
       </c>
-      <c r="E106" s="22" t="inlineStr">
+      <c r="E106" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F106" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G106" s="23" t="n">
+      <c r="F106" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" s="40" t="n">
         <v>1363734.16</v>
       </c>
-      <c r="H106" s="23" t="n">
+      <c r="H106" s="40" t="n">
         <v>-32302.86</v>
       </c>
-      <c r="I106" s="23" t="n">
+      <c r="I106" s="40" t="n">
         <v>1331431.3</v>
       </c>
-      <c r="J106" s="22" t="inlineStr">
+      <c r="J106" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K106" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L106" s="23" t="n">
+      <c r="K106" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L106" s="40" t="n">
         <v>-31801.37</v>
       </c>
-      <c r="M106" s="23" t="n">
+      <c r="M106" s="40" t="n">
         <v>1331455.9</v>
       </c>
-      <c r="N106" s="23" t="n">
+      <c r="N106" s="40" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="O106" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P106" s="23" t="n">
+      <c r="O106" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P106" s="40" t="n">
         <v>501.49</v>
       </c>
-      <c r="Q106" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" s="23" t="n">
+      <c r="Q106" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" s="40" t="n">
         <v>-24.6</v>
       </c>
-      <c r="S106" s="23" t="n">
+      <c r="S106" s="40" t="n">
         <v>476.82</v>
       </c>
-      <c r="T106" s="22" t="inlineStr">
+      <c r="T106" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U106" s="22" t="inlineStr">
+      <c r="U106" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V106" s="22" t="inlineStr">
+      <c r="V106" s="39" t="inlineStr">
         <is>
           <t>143000</t>
         </is>
       </c>
-      <c r="W106" s="22" t="inlineStr">
+      <c r="W106" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">MLD     </t>
         </is>
       </c>
+      <c r="X106" s="41" t="n"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11261,95 +11951,96 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="22" t="inlineStr">
+      <c r="A119" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B119" s="22" t="inlineStr">
+      <c r="B119" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C119" s="22" t="inlineStr">
+      <c r="C119" s="39" t="inlineStr">
         <is>
           <t>00223925</t>
         </is>
       </c>
-      <c r="D119" s="22" t="inlineStr">
+      <c r="D119" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143000.PRS           </t>
         </is>
       </c>
-      <c r="E119" s="22" t="inlineStr">
+      <c r="E119" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F119" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G119" s="23" t="n">
+      <c r="F119" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" s="40" t="n">
         <v>1403485.38</v>
       </c>
-      <c r="H119" s="23" t="n">
+      <c r="H119" s="40" t="n">
         <v>-85744.08</v>
       </c>
-      <c r="I119" s="23" t="n">
+      <c r="I119" s="40" t="n">
         <v>1317741.3</v>
       </c>
-      <c r="J119" s="22" t="inlineStr">
+      <c r="J119" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K119" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L119" s="23" t="n">
+      <c r="K119" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L119" s="40" t="n">
         <v>-85379.74000000001</v>
       </c>
-      <c r="M119" s="23" t="n">
+      <c r="M119" s="40" t="n">
         <v>1245693.62</v>
       </c>
-      <c r="N119" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O119" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P119" s="23" t="n">
+      <c r="N119" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O119" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P119" s="40" t="n">
         <v>364.34</v>
       </c>
-      <c r="Q119" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R119" s="23" t="n">
+      <c r="Q119" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R119" s="40" t="n">
         <v>72047.67999999999</v>
       </c>
-      <c r="S119" s="23" t="n">
+      <c r="S119" s="40" t="n">
         <v>72412.02</v>
       </c>
-      <c r="T119" s="22" t="inlineStr">
+      <c r="T119" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U119" s="22" t="inlineStr">
+      <c r="U119" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V119" s="22" t="inlineStr">
+      <c r="V119" s="39" t="inlineStr">
         <is>
           <t>143000</t>
         </is>
       </c>
-      <c r="W119" s="22" t="inlineStr">
+      <c r="W119" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">PRS     </t>
         </is>
       </c>
+      <c r="X119" s="41" t="n"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -12444,95 +13135,96 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="22" t="inlineStr">
+      <c r="A132" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B132" s="22" t="inlineStr">
+      <c r="B132" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C132" s="22" t="inlineStr">
+      <c r="C132" s="39" t="inlineStr">
         <is>
           <t>00223933</t>
         </is>
       </c>
-      <c r="D132" s="22" t="inlineStr">
+      <c r="D132" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143000.S/A           </t>
         </is>
       </c>
-      <c r="E132" s="22" t="inlineStr">
+      <c r="E132" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F132" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G132" s="23" t="n">
+      <c r="F132" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G132" s="40" t="n">
         <v>669415.85</v>
       </c>
-      <c r="H132" s="23" t="n">
+      <c r="H132" s="40" t="n">
         <v>50174.75</v>
       </c>
-      <c r="I132" s="23" t="n">
+      <c r="I132" s="40" t="n">
         <v>719590.6</v>
       </c>
-      <c r="J132" s="22" t="inlineStr">
+      <c r="J132" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K132" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L132" s="23" t="n">
+      <c r="K132" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L132" s="40" t="n">
         <v>52245.7</v>
       </c>
-      <c r="M132" s="23" t="n">
+      <c r="M132" s="40" t="n">
         <v>722116.0600000001</v>
       </c>
-      <c r="N132" s="23" t="n">
+      <c r="N132" s="40" t="n">
         <v>-0.03</v>
       </c>
-      <c r="O132" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P132" s="23" t="n">
+      <c r="O132" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P132" s="40" t="n">
         <v>2070.95</v>
       </c>
-      <c r="Q132" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R132" s="23" t="n">
+      <c r="Q132" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R132" s="40" t="n">
         <v>-2525.46</v>
       </c>
-      <c r="S132" s="23" t="n">
+      <c r="S132" s="40" t="n">
         <v>-454.48</v>
       </c>
-      <c r="T132" s="22" t="inlineStr">
+      <c r="T132" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U132" s="22" t="inlineStr">
+      <c r="U132" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V132" s="22" t="inlineStr">
+      <c r="V132" s="39" t="inlineStr">
         <is>
           <t>143000</t>
         </is>
       </c>
-      <c r="W132" s="22" t="inlineStr">
+      <c r="W132" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">S/A     </t>
         </is>
       </c>
+      <c r="X132" s="41" t="n"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -13627,95 +14319,96 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="22" t="inlineStr">
+      <c r="A145" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B145" s="22" t="inlineStr">
+      <c r="B145" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C145" s="22" t="inlineStr">
+      <c r="C145" s="39" t="inlineStr">
         <is>
           <t>00223941</t>
         </is>
       </c>
-      <c r="D145" s="22" t="inlineStr">
+      <c r="D145" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143000.S/C           </t>
         </is>
       </c>
-      <c r="E145" s="22" t="inlineStr">
+      <c r="E145" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F145" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G145" s="23" t="n">
+      <c r="F145" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G145" s="40" t="n">
         <v>902555.2</v>
       </c>
-      <c r="H145" s="23" t="n">
+      <c r="H145" s="40" t="n">
         <v>1096.21</v>
       </c>
-      <c r="I145" s="23" t="n">
+      <c r="I145" s="40" t="n">
         <v>903651.41</v>
       </c>
-      <c r="J145" s="22" t="inlineStr">
+      <c r="J145" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K145" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L145" s="23" t="n">
+      <c r="K145" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L145" s="40" t="n">
         <v>1352.56</v>
       </c>
-      <c r="M145" s="23" t="n">
+      <c r="M145" s="40" t="n">
         <v>909036.22</v>
       </c>
-      <c r="N145" s="23" t="n">
+      <c r="N145" s="40" t="n">
         <v>-0.01</v>
       </c>
-      <c r="O145" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P145" s="23" t="n">
+      <c r="O145" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P145" s="40" t="n">
         <v>256.35</v>
       </c>
-      <c r="Q145" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R145" s="23" t="n">
+      <c r="Q145" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R145" s="40" t="n">
         <v>-5384.81</v>
       </c>
-      <c r="S145" s="23" t="n">
+      <c r="S145" s="40" t="n">
         <v>-5128.45</v>
       </c>
-      <c r="T145" s="22" t="inlineStr">
+      <c r="T145" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U145" s="22" t="inlineStr">
+      <c r="U145" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V145" s="22" t="inlineStr">
+      <c r="V145" s="39" t="inlineStr">
         <is>
           <t>143000</t>
         </is>
       </c>
-      <c r="W145" s="22" t="inlineStr">
+      <c r="W145" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">S/C     </t>
         </is>
       </c>
+      <c r="X145" s="41" t="n"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -14810,95 +15503,96 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="22" t="inlineStr">
+      <c r="A158" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B158" s="22" t="inlineStr">
+      <c r="B158" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C158" s="22" t="inlineStr">
+      <c r="C158" s="39" t="inlineStr">
         <is>
           <t>00223950</t>
         </is>
       </c>
-      <c r="D158" s="22" t="inlineStr">
+      <c r="D158" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143000.SEC           </t>
         </is>
       </c>
-      <c r="E158" s="22" t="inlineStr">
+      <c r="E158" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F158" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G158" s="23" t="n">
+      <c r="F158" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G158" s="40" t="n">
         <v>75889.22</v>
       </c>
-      <c r="H158" s="23" t="n">
+      <c r="H158" s="40" t="n">
         <v>31234.87</v>
       </c>
-      <c r="I158" s="23" t="n">
+      <c r="I158" s="40" t="n">
         <v>107124.09</v>
       </c>
-      <c r="J158" s="22" t="inlineStr">
+      <c r="J158" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K158" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L158" s="23" t="n">
+      <c r="K158" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" s="40" t="n">
         <v>31903.75</v>
       </c>
-      <c r="M158" s="23" t="n">
+      <c r="M158" s="40" t="n">
         <v>175328.95</v>
       </c>
-      <c r="N158" s="23" t="n">
+      <c r="N158" s="40" t="n">
         <v>-0.03</v>
       </c>
-      <c r="O158" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P158" s="23" t="n">
+      <c r="O158" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P158" s="40" t="n">
         <v>668.88</v>
       </c>
-      <c r="Q158" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R158" s="23" t="n">
+      <c r="Q158" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R158" s="40" t="n">
         <v>-68204.86</v>
       </c>
-      <c r="S158" s="23" t="n">
+      <c r="S158" s="40" t="n">
         <v>-67535.95</v>
       </c>
-      <c r="T158" s="22" t="inlineStr">
+      <c r="T158" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U158" s="22" t="inlineStr">
+      <c r="U158" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V158" s="22" t="inlineStr">
+      <c r="V158" s="39" t="inlineStr">
         <is>
           <t>143000</t>
         </is>
       </c>
-      <c r="W158" s="22" t="inlineStr">
+      <c r="W158" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">SEC     </t>
         </is>
       </c>
+      <c r="X158" s="41" t="n"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -15993,95 +16687,96 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="22" t="inlineStr">
+      <c r="A171" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B171" s="22" t="inlineStr">
+      <c r="B171" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C171" s="22" t="inlineStr">
+      <c r="C171" s="39" t="inlineStr">
         <is>
           <t>00832510</t>
         </is>
       </c>
-      <c r="D171" s="22" t="inlineStr">
+      <c r="D171" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.143100               </t>
         </is>
       </c>
-      <c r="E171" s="22" t="inlineStr">
+      <c r="E171" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F171" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G171" s="23" t="n">
+      <c r="F171" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G171" s="40" t="n">
         <v>173488.5</v>
       </c>
-      <c r="H171" s="23" t="n">
+      <c r="H171" s="40" t="n">
         <v>10953.42</v>
       </c>
-      <c r="I171" s="23" t="n">
+      <c r="I171" s="40" t="n">
         <v>184441.92</v>
       </c>
-      <c r="J171" s="22" t="inlineStr">
+      <c r="J171" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K171" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L171" s="23" t="n">
+      <c r="K171" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" s="40" t="n">
         <v>10953.42</v>
       </c>
-      <c r="M171" s="23" t="n">
+      <c r="M171" s="40" t="n">
         <v>184445.09</v>
       </c>
-      <c r="N171" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O171" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P171" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q171" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R171" s="23" t="n">
+      <c r="N171" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O171" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P171" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q171" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R171" s="40" t="n">
         <v>-3.17</v>
       </c>
-      <c r="S171" s="23" t="n">
+      <c r="S171" s="40" t="n">
         <v>-3.17</v>
       </c>
-      <c r="T171" s="22" t="inlineStr">
+      <c r="T171" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U171" s="22" t="inlineStr">
+      <c r="U171" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V171" s="22" t="inlineStr">
+      <c r="V171" s="39" t="inlineStr">
         <is>
           <t>143100</t>
         </is>
       </c>
-      <c r="W171" s="22" t="inlineStr">
+      <c r="W171" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
+      <c r="X171" s="41" t="n"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -17176,95 +17871,96 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="22" t="inlineStr">
+      <c r="A184" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B184" s="22" t="inlineStr">
+      <c r="B184" s="39" t="inlineStr">
         <is>
           <t>00010</t>
         </is>
       </c>
-      <c r="C184" s="22" t="inlineStr">
+      <c r="C184" s="39" t="inlineStr">
         <is>
           <t>00223976</t>
         </is>
       </c>
-      <c r="D184" s="22" t="inlineStr">
+      <c r="D184" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">1000000.145000               </t>
         </is>
       </c>
-      <c r="E184" s="22" t="inlineStr">
+      <c r="E184" s="39" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F184" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G184" s="23" t="n">
+      <c r="F184" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G184" s="40" t="n">
         <v>2177917.09</v>
       </c>
-      <c r="H184" s="23" t="n">
+      <c r="H184" s="40" t="n">
         <v>-35817.56</v>
       </c>
-      <c r="I184" s="23" t="n">
+      <c r="I184" s="40" t="n">
         <v>2142099.53</v>
       </c>
-      <c r="J184" s="22" t="inlineStr">
+      <c r="J184" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K184" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L184" s="23" t="n">
+      <c r="K184" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L184" s="40" t="n">
         <v>-35099.3</v>
       </c>
-      <c r="M184" s="23" t="n">
+      <c r="M184" s="40" t="n">
         <v>2113141.74</v>
       </c>
-      <c r="N184" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O184" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P184" s="23" t="n">
+      <c r="N184" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O184" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P184" s="40" t="n">
         <v>-2729.77</v>
       </c>
-      <c r="Q184" s="23" t="n">
+      <c r="Q184" s="40" t="n">
         <v>-3448.03</v>
       </c>
-      <c r="R184" s="23" t="n">
+      <c r="R184" s="40" t="n">
         <v>28957.79</v>
       </c>
-      <c r="S184" s="23" t="n">
+      <c r="S184" s="40" t="n">
         <v>29676.05</v>
       </c>
-      <c r="T184" s="22" t="inlineStr">
+      <c r="T184" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U184" s="22" t="inlineStr">
+      <c r="U184" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     1000000</t>
         </is>
       </c>
-      <c r="V184" s="22" t="inlineStr">
+      <c r="V184" s="39" t="inlineStr">
         <is>
           <t>145000</t>
         </is>
       </c>
-      <c r="W184" s="22" t="inlineStr">
+      <c r="W184" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
+      <c r="X184" s="41" t="n"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -18359,95 +19055,96 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="22" t="inlineStr">
+      <c r="A197" s="39" t="inlineStr">
         <is>
           <t>2016-08-27</t>
         </is>
       </c>
-      <c r="B197" s="22" t="inlineStr">
+      <c r="B197" s="39" t="inlineStr">
         <is>
           <t>00050</t>
         </is>
       </c>
-      <c r="C197" s="22" t="inlineStr">
+      <c r="C197" s="39" t="inlineStr">
         <is>
           <t>00883173</t>
         </is>
       </c>
-      <c r="D197" s="22" t="inlineStr">
+      <c r="D197" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">5000000.145000               </t>
         </is>
       </c>
-      <c r="E197" s="22" t="inlineStr">
+      <c r="E197" s="39" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="F197" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G197" s="23" t="n">
+      <c r="F197" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G197" s="40" t="n">
         <v>1343597.6</v>
       </c>
-      <c r="H197" s="23" t="n">
+      <c r="H197" s="40" t="n">
         <v>35981.17</v>
       </c>
-      <c r="I197" s="23" t="n">
+      <c r="I197" s="40" t="n">
         <v>1379578.77</v>
       </c>
-      <c r="J197" s="22" t="inlineStr">
+      <c r="J197" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end     </t>
         </is>
       </c>
-      <c r="K197" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L197" s="23" t="n">
+      <c r="K197" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L197" s="40" t="n">
         <v>35828.26</v>
       </c>
-      <c r="M197" s="23" t="n">
+      <c r="M197" s="40" t="n">
         <v>1404782.47</v>
       </c>
-      <c r="N197" s="23" t="n">
+      <c r="N197" s="40" t="n">
         <v>-18674.74</v>
       </c>
-      <c r="O197" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P197" s="23" t="n">
+      <c r="O197" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P197" s="40" t="n">
         <v>-152.91</v>
       </c>
-      <c r="Q197" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="R197" s="23" t="n">
+      <c r="Q197" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R197" s="40" t="n">
         <v>-25203.7</v>
       </c>
-      <c r="S197" s="23" t="n">
+      <c r="S197" s="40" t="n">
         <v>-6681.87</v>
       </c>
-      <c r="T197" s="22" t="inlineStr">
+      <c r="T197" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">end - Nov 16 2023 11:51AM     </t>
         </is>
       </c>
-      <c r="U197" s="22" t="inlineStr">
+      <c r="U197" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">     5000000</t>
         </is>
       </c>
-      <c r="V197" s="22" t="inlineStr">
+      <c r="V197" s="39" t="inlineStr">
         <is>
           <t>145000</t>
         </is>
       </c>
-      <c r="W197" s="22" t="inlineStr">
+      <c r="W197" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
+      <c r="X197" s="41" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:X2"/>
@@ -18457,614 +19154,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C44"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.625" defaultRowHeight="15.75"/>
-  <cols>
-    <col width="28" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="52" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>REPORT SUMMARY</t>
-        </is>
-      </c>
-      <c r="B1" s="25" t="n"/>
-      <c r="C1" s="25" t="n"/>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Report Generated</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Wednesday, April 22, 2026, 5:21 PM</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n"/>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Current (End) Period</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>2016-08-27</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Most recent period in dataset</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Dataset Period Range</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>2015-08-29 through 2016-08-27</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>13 fiscal periods</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>GLOK Baseline Period</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>2015-08-29</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Earliest period loaded</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>VarOK Baseline Date</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>2021-05-27 13:07:51</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Date RapidReconciler was last reset</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Companies</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>2 (00010, 00050)</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Co. 10 = 14 accounts; Co. 50 = 1 account</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Accounts (Unique)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Distinct LongAccount values</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Total Data Rows</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>195</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>15 accounts x 13 periods</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>GLOK = "no" Rows</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>No GL roll forward breaks detected</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>VarOK = "no" Rows</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>No variance roll forward breaks detected</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>End Period Total EndGL</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>$18,724,064.22</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Sum of all accounts, current period</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>End Period Total Perpetual</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>$18,710,860.69</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Sum of all accounts, current period</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>End Period UnpostBatch</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>No unposted batches in current period</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="25" t="n"/>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="25" t="n"/>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>ROW COLOR KEY</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="n"/>
-      <c r="C17" s="25" t="n"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Criteria</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Row Count</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="26" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>GLOK = "no" OR VarOK = "no" — roll forward break</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="27" t="inlineStr">
-        <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>GLOK = "end" with non-zero UnpostBatch</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
-        <is>
-          <t>Yellow</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>GLOK = "end" with zero UnpostBatch — current period, clean</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
-        <is>
-          <t>Blue</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>GLOK = "yes" with non-zero UnpostBatch — historical with pending batches</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>White/Gray</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>All other rows (baseline or clean historical)</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>180</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="25" t="n"/>
-      <c r="B24" s="25" t="n"/>
-      <c r="C24" s="25" t="n"/>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>GL ROLL FORWARD (GLOK) FINDINGS</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="n"/>
-      <c r="C25" s="25" t="n"/>
-    </row>
-    <row r="26" ht="140" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>No GLOK = "no" rows were found in this export. All 195 rows carry the baseline, yes, or end designation. The GL balance rolled forward without interruption across all 13 periods for all 15 accounts in both companies. No corrective action is required for GL continuity.</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="25" t="n"/>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="25" t="n"/>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="25" t="n"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>VARIANCE ROLL FORWARD (VarOK) FINDINGS</t>
-        </is>
-      </c>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="25" t="n"/>
-    </row>
-    <row r="29" ht="140" customHeight="1">
-      <c r="A29" s="19" t="inlineStr">
-        <is>
-          <t>No VarOK = "no" rows were found in this export. The variance chain is intact across all periods for all accounts. The VarOK baseline date (2021-05-27) post-dating the dataset start (2015-08-29) is expected — it reflects a RapidReconciler reset after initial data load.</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="25" t="n"/>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>HISTORICAL UNPOSTED BATCH SUMMARY</t>
-        </is>
-      </c>
-      <c r="B31" s="25" t="n"/>
-      <c r="C31" s="25" t="n"/>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>LongAccount</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>EndGL | UnpostBatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>No accounts in any historical period have a non-zero UnpostBatch.</t>
-        </is>
-      </c>
-      <c r="B33" s="25" t="n"/>
-      <c r="C33" s="25" t="n"/>
-    </row>
-    <row r="34" ht="154" customHeight="1">
-      <c r="A34" s="19" t="inlineStr">
-        <is>
-          <t>Covers all periods except the current (end) period. A non-zero UnpostBatch in a historical period indicates a batch was approved but unposted at period-end and posted retroactively, which would have caused GLOK = "no" in the following period. In this export no historical unposted batches are present.</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="n"/>
-      <c r="C34" s="25" t="n"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="25" t="n"/>
-      <c r="B35" s="25" t="n"/>
-      <c r="C35" s="25" t="n"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>PERIOD VARIANCE BY ACCOUNT</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="n"/>
-      <c r="C36" s="25" t="n"/>
-    </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>LongAccount</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Variance | OOB | UnpostBatch</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>5000000.145000</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>2016-07-30</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Var: -$262.43  OOB: -$18,674.74  UnpostBatch: $0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="154" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Covers the prior 3 periods only (2016-05-28, 2016-07-02, 2016-07-30). Rows are shown where OOB absolute value exceeds $100 or UnpostBatch is non-zero. JE amounts and CardexVar are excluded from this section. OOB in these periods is informational; escalate only if accompanied by a VarOK = "no" flag.</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="n"/>
-      <c r="C39" s="25" t="n"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="25" t="n"/>
-      <c r="B40" s="25" t="n"/>
-      <c r="C40" s="25" t="n"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>RECOMMENDED ACTIONS</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="n"/>
-      <c r="C41" s="25" t="n"/>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="112" customHeight="1">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t>1 — High</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>Investigate OOB on 5000000.145000 (Company 50, GBP) in 2016-07-30: OOB of -$18,674.74 exceeds the $100 threshold in a closed historical period. Query F0902 and F0911 for this account and period to confirm the discrepancy. If confirmed, run R099102 in proof mode then final mode to resync F0902 from F0911. Involve your JD Edwards administrator before running in final mode.</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>Cost Accountant / JD Edwards Administrator</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="70" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>2 — Informational</t>
-        </is>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
-        <is>
-          <t>No GL roll forward breaks (GLOK = "no") and no variance roll forward breaks (VarOK = "no") were detected. No batch posting or R099102 is required for continuity. Confirm this remains true at the next RapidReconciler refresh.</t>
-        </is>
-      </c>
-      <c r="C44" s="16" t="inlineStr">
-        <is>
-          <t>Cost Accountant</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A26:C26"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>